<commit_message>
added exist check and changed test data
</commit_message>
<xml_diff>
--- a/rules/CORE-002008/positive/01/data/CORE-002008-positive-01.xlsx
+++ b/rules/CORE-002008/positive/01/data/CORE-002008-positive-01.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/positive/01/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/CORE-002008/positive/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7DBC523-E00B-AD43-9CF3-C3D304F8C972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DA1347-1586-E440-ACBE-C49261071DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="660" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{2322A04D-5CB7-449F-8225-CADE54871F75}"/>
+    <workbookView xWindow="1500" yWindow="660" windowWidth="28740" windowHeight="18980" activeTab="2" xr2:uid="{2322A04D-5CB7-449F-8225-CADE54871F75}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="8" r:id="rId1"/>
     <sheet name="Datasets" sheetId="9" r:id="rId2"/>
-    <sheet name="mh.xpt" sheetId="10" r:id="rId3"/>
-    <sheet name="ae.xpt" sheetId="4" r:id="rId4"/>
+    <sheet name="ae.xpt" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="104">
   <si>
     <t>STUDYID</t>
   </si>
@@ -320,9 +319,6 @@
     <t>2019-03-16</t>
   </si>
   <si>
-    <t>Injury, poisoning and procedural complications</t>
-  </si>
-  <si>
     <t>Product</t>
   </si>
   <si>
@@ -335,36 +331,6 @@
     <t>3-4</t>
   </si>
   <si>
-    <t>Category for Medical History</t>
-  </si>
-  <si>
-    <t>Reported Term for the Medical History</t>
-  </si>
-  <si>
-    <t>Start Date/Time of Medical History Event</t>
-  </si>
-  <si>
-    <t>Study Day of Start of Observation</t>
-  </si>
-  <si>
-    <t>CDISCPILOT01</t>
-  </si>
-  <si>
-    <t>MH</t>
-  </si>
-  <si>
-    <t>CDISC010</t>
-  </si>
-  <si>
-    <t>GENERAL</t>
-  </si>
-  <si>
-    <t>CDISC011</t>
-  </si>
-  <si>
-    <t>CDISC012</t>
-  </si>
-  <si>
     <t>Filename</t>
   </si>
   <si>
@@ -381,168 +347,6 @@
   </si>
   <si>
     <t>Adverse Events</t>
-  </si>
-  <si>
-    <t>Allergic conditions</t>
-  </si>
-  <si>
-    <t>MEDICAL HISTORY</t>
-  </si>
-  <si>
-    <t>IMMUNE SYSTEM DISORDERS</t>
-  </si>
-  <si>
-    <t>Immune system disorders</t>
-  </si>
-  <si>
-    <t>SURGICAL HISTORY</t>
-  </si>
-  <si>
-    <t>Surgical and medical procedures</t>
-  </si>
-  <si>
-    <t>Bone and joint injuries</t>
-  </si>
-  <si>
-    <t>MUSCULOSKELETAL AND CONNECTIVE TISSUE DISORDERS</t>
-  </si>
-  <si>
-    <t>REPRODUCTIVE SYSTEM AND BREAST DISORDERS</t>
-  </si>
-  <si>
-    <t>Menopause</t>
-  </si>
-  <si>
-    <t>Age related issues</t>
-  </si>
-  <si>
-    <t>Age related factors</t>
-  </si>
-  <si>
-    <t>Social circumstances</t>
-  </si>
-  <si>
-    <t>MHSEQ</t>
-  </si>
-  <si>
-    <t>MHTERM</t>
-  </si>
-  <si>
-    <t>MHLLT</t>
-  </si>
-  <si>
-    <t>MHLLTCD</t>
-  </si>
-  <si>
-    <t>MHDECOD</t>
-  </si>
-  <si>
-    <t>MHPTCD</t>
-  </si>
-  <si>
-    <t>MHHLT</t>
-  </si>
-  <si>
-    <t>MHHLTCD</t>
-  </si>
-  <si>
-    <t>MHHLGT</t>
-  </si>
-  <si>
-    <t>MHHLGTCD</t>
-  </si>
-  <si>
-    <t>MHCAT</t>
-  </si>
-  <si>
-    <t>MHBODSYS</t>
-  </si>
-  <si>
-    <t>MHBDSYCD</t>
-  </si>
-  <si>
-    <t>MHSOC</t>
-  </si>
-  <si>
-    <t>MHSOCCD</t>
-  </si>
-  <si>
-    <t>MHSTDTC</t>
-  </si>
-  <si>
-    <t>MHSTDY</t>
-  </si>
-  <si>
-    <t>MENOPAUSE</t>
-  </si>
-  <si>
-    <t>Bone and joint therapeutic procedures</t>
-  </si>
-  <si>
-    <t>Joint therapeutic procedures</t>
-  </si>
-  <si>
-    <t>KNEE SURGERY NOS</t>
-  </si>
-  <si>
-    <t>Knee surgery NOS</t>
-  </si>
-  <si>
-    <t>Knee operation</t>
-  </si>
-  <si>
-    <t>NICKEL ALLERGY</t>
-  </si>
-  <si>
-    <t>Allergy to metals</t>
-  </si>
-  <si>
-    <t>Allergic conditions NEC</t>
-  </si>
-  <si>
-    <t>SHOULDER DISLOCATION</t>
-  </si>
-  <si>
-    <t>Shoulder dislocation</t>
-  </si>
-  <si>
-    <t>Joint dislocation</t>
-  </si>
-  <si>
-    <t>Fractures and dislocations NEC</t>
-  </si>
-  <si>
-    <t>2025-01-12</t>
-  </si>
-  <si>
-    <t>2025-01-13</t>
-  </si>
-  <si>
-    <t>2025-01-14</t>
-  </si>
-  <si>
-    <t>2025-01-15</t>
-  </si>
-  <si>
-    <t>2025-01-16</t>
-  </si>
-  <si>
-    <t>-8</t>
-  </si>
-  <si>
-    <t>-9</t>
-  </si>
-  <si>
-    <t>-10</t>
-  </si>
-  <si>
-    <t>-11</t>
-  </si>
-  <si>
-    <t>-12</t>
-  </si>
-  <si>
-    <t>Nickel allergy</t>
   </si>
   <si>
     <t>Upset stomach</t>
@@ -552,22 +356,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -583,14 +372,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -599,17 +382,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -629,21 +407,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -702,83 +465,44 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="1" builtinId="10"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <i/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <i/>
@@ -1121,18 +845,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1150,27 +874,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>109</v>
+      <c r="A1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>111</v>
+      <c r="A2" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>113</v>
+      <c r="A3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1179,602 +903,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7C8696D-62B8-4685-B451-7EC2CDC82766}">
-  <dimension ref="A1:T9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.5" customWidth="1"/>
-    <col min="2" max="2" width="16.1640625" customWidth="1"/>
-    <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="32.33203125" customWidth="1"/>
-    <col min="5" max="5" width="23.6640625" customWidth="1"/>
-    <col min="6" max="6" width="31.6640625" customWidth="1"/>
-    <col min="7" max="7" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.33203125" customWidth="1"/>
-    <col min="10" max="10" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="52.1640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="43.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="44.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="20.6640625" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q1" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="R1" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="S1" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="T1" s="7" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" ht="48" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
-        <v>12</v>
-      </c>
-      <c r="B4" s="3">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3">
-        <v>8</v>
-      </c>
-      <c r="D4" s="3">
-        <v>8</v>
-      </c>
-      <c r="E4" s="4">
-        <v>50</v>
-      </c>
-      <c r="F4" s="3">
-        <v>19</v>
-      </c>
-      <c r="G4" s="3">
-        <v>38</v>
-      </c>
-      <c r="H4" s="3">
-        <v>8</v>
-      </c>
-      <c r="I4" s="3">
-        <v>38</v>
-      </c>
-      <c r="J4" s="3">
-        <v>8</v>
-      </c>
-      <c r="K4" s="3">
-        <v>65</v>
-      </c>
-      <c r="L4" s="3">
-        <v>8</v>
-      </c>
-      <c r="M4" s="3">
-        <v>55</v>
-      </c>
-      <c r="N4" s="3">
-        <v>8</v>
-      </c>
-      <c r="O4" s="3">
-        <v>52</v>
-      </c>
-      <c r="P4" s="3">
-        <v>8</v>
-      </c>
-      <c r="Q4" s="3">
-        <v>52</v>
-      </c>
-      <c r="R4" s="3">
-        <v>8</v>
-      </c>
-      <c r="S4" s="1">
-        <v>10</v>
-      </c>
-      <c r="T4" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D5" s="1">
-        <v>1</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F5" t="s">
-        <v>147</v>
-      </c>
-      <c r="G5" t="s">
-        <v>148</v>
-      </c>
-      <c r="H5">
-        <v>10049662</v>
-      </c>
-      <c r="I5" t="s">
-        <v>149</v>
-      </c>
-      <c r="J5">
-        <v>10049548</v>
-      </c>
-      <c r="K5" t="s">
-        <v>146</v>
-      </c>
-      <c r="L5">
-        <v>10023221</v>
-      </c>
-      <c r="M5" t="s">
-        <v>145</v>
-      </c>
-      <c r="N5">
-        <v>10005944</v>
-      </c>
-      <c r="O5" t="s">
-        <v>118</v>
-      </c>
-      <c r="P5" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>119</v>
-      </c>
-      <c r="R5">
-        <v>10042613</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C6" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="1">
-        <v>1</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F6" t="s">
-        <v>147</v>
-      </c>
-      <c r="G6" t="s">
-        <v>148</v>
-      </c>
-      <c r="H6">
-        <v>10049662</v>
-      </c>
-      <c r="I6" t="s">
-        <v>149</v>
-      </c>
-      <c r="J6">
-        <v>10049548</v>
-      </c>
-      <c r="K6" t="s">
-        <v>146</v>
-      </c>
-      <c r="L6">
-        <v>10023221</v>
-      </c>
-      <c r="M6" t="s">
-        <v>145</v>
-      </c>
-      <c r="N6">
-        <v>10005944</v>
-      </c>
-      <c r="O6" t="s">
-        <v>118</v>
-      </c>
-      <c r="P6" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>119</v>
-      </c>
-      <c r="R6">
-        <v>10042613</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D7" s="1">
-        <v>1</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F7" t="s">
-        <v>144</v>
-      </c>
-      <c r="G7" t="s">
-        <v>123</v>
-      </c>
-      <c r="H7">
-        <v>10027308</v>
-      </c>
-      <c r="I7" t="s">
-        <v>123</v>
-      </c>
-      <c r="J7">
-        <v>10027308</v>
-      </c>
-      <c r="K7" t="s">
-        <v>124</v>
-      </c>
-      <c r="L7">
-        <v>10001475</v>
-      </c>
-      <c r="M7" t="s">
-        <v>125</v>
-      </c>
-      <c r="N7">
-        <v>10001474</v>
-      </c>
-      <c r="O7" t="s">
-        <v>115</v>
-      </c>
-      <c r="P7" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>126</v>
-      </c>
-      <c r="R7">
-        <v>10041244</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="1">
-        <v>1</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F8" t="s">
-        <v>150</v>
-      </c>
-      <c r="G8" t="s">
-        <v>167</v>
-      </c>
-      <c r="H8">
-        <v>10088472</v>
-      </c>
-      <c r="I8" t="s">
-        <v>151</v>
-      </c>
-      <c r="J8">
-        <v>10066414</v>
-      </c>
-      <c r="K8" t="s">
-        <v>152</v>
-      </c>
-      <c r="L8">
-        <v>10027654</v>
-      </c>
-      <c r="M8" t="s">
-        <v>114</v>
-      </c>
-      <c r="N8">
-        <v>10001708</v>
-      </c>
-      <c r="O8" t="s">
-        <v>115</v>
-      </c>
-      <c r="P8" t="s">
-        <v>116</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>117</v>
-      </c>
-      <c r="R8">
-        <v>10021428</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F9" t="s">
-        <v>153</v>
-      </c>
-      <c r="G9" t="s">
-        <v>154</v>
-      </c>
-      <c r="H9">
-        <v>10040612</v>
-      </c>
-      <c r="I9" t="s">
-        <v>155</v>
-      </c>
-      <c r="J9">
-        <v>10023204</v>
-      </c>
-      <c r="K9" t="s">
-        <v>156</v>
-      </c>
-      <c r="L9">
-        <v>10027677</v>
-      </c>
-      <c r="M9" t="s">
-        <v>120</v>
-      </c>
-      <c r="N9">
-        <v>10005942</v>
-      </c>
-      <c r="O9" t="s">
-        <v>118</v>
-      </c>
-      <c r="P9" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>93</v>
-      </c>
-      <c r="R9">
-        <v>10022117</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>166</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A2:T4">
-    <cfRule type="notContainsBlanks" dxfId="1" priority="1">
-      <formula>LEN(TRIM(A2))&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63135780-15D4-4B3D-9F00-D6DA3A668942}">
   <dimension ref="A1:AA10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1785,334 +913,334 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="W1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="X1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Y1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="Z1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="AA1" s="10" t="s">
+      <c r="AA1" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="32" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="J2" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="L2" s="11" t="s">
+      <c r="L2" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="M2" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="N2" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="O2" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="P2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="R2" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="S2" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="T2" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="U2" s="11" t="s">
+      <c r="U2" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="V2" s="11" t="s">
+      <c r="V2" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="W2" s="11" t="s">
+      <c r="W2" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="X2" s="11" t="s">
+      <c r="X2" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="Y2" s="11" t="s">
+      <c r="Y2" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="Z2" s="11" t="s">
+      <c r="Z2" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="AA2" s="12" t="s">
+      <c r="AA2" s="8" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="13" t="s">
+      <c r="A3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="13" t="s">
+      <c r="E3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="J3" s="13" t="s">
+      <c r="I3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="L3" s="13" t="s">
+      <c r="K3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="L3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="N3" s="13" t="s">
+      <c r="M3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="N3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="P3" s="13" t="s">
+      <c r="O3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="P3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="R3" s="13" t="s">
+      <c r="Q3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="R3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="S3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="T3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="U3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="V3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="W3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="X3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="Y3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="Z3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="AA3" s="14" t="s">
+      <c r="S3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="U3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="V3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="W3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA3" s="10" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A4" s="11">
+      <c r="A4" s="7">
         <v>10</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="7">
         <v>2</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="7">
         <v>14</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="7">
         <v>8</v>
       </c>
-      <c r="E4" s="11">
-        <v>4</v>
-      </c>
-      <c r="F4" s="11">
+      <c r="E4" s="7">
+        <v>4</v>
+      </c>
+      <c r="F4" s="7">
         <v>38</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="7">
         <v>38</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="7">
         <v>8</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="7">
         <v>38</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="7">
         <v>8</v>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="7">
         <v>65</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="7">
         <v>8</v>
       </c>
-      <c r="M4" s="11">
+      <c r="M4" s="7">
         <v>55</v>
       </c>
-      <c r="N4" s="11">
+      <c r="N4" s="7">
         <v>8</v>
       </c>
-      <c r="O4" s="11">
+      <c r="O4" s="7">
         <v>52</v>
       </c>
-      <c r="P4" s="11">
+      <c r="P4" s="7">
         <v>8</v>
       </c>
-      <c r="Q4" s="11">
+      <c r="Q4" s="7">
         <v>52</v>
       </c>
-      <c r="R4" s="11">
+      <c r="R4" s="7">
         <v>8</v>
       </c>
-      <c r="S4" s="11">
+      <c r="S4" s="7">
         <v>8</v>
       </c>
-      <c r="T4" s="11">
+      <c r="T4" s="7">
         <v>1</v>
       </c>
-      <c r="U4" s="11">
+      <c r="U4" s="7">
         <v>1</v>
       </c>
-      <c r="V4" s="11">
+      <c r="V4" s="7">
         <v>1</v>
       </c>
-      <c r="W4" s="11">
+      <c r="W4" s="7">
         <v>26</v>
       </c>
-      <c r="X4" s="11">
+      <c r="X4" s="7">
         <v>1</v>
       </c>
-      <c r="Y4" s="11">
+      <c r="Y4" s="7">
         <v>10</v>
       </c>
-      <c r="Z4" s="11">
+      <c r="Z4" s="7">
         <v>1</v>
       </c>
-      <c r="AA4" s="12">
+      <c r="AA4" s="8">
         <v>8</v>
       </c>
     </row>
@@ -2136,7 +1264,7 @@
         <v>70</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>168</v>
+        <v>103</v>
       </c>
       <c r="H5" s="1">
         <v>10046318</v>
@@ -2210,7 +1338,7 @@
         <v>70</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>168</v>
+        <v>103</v>
       </c>
       <c r="H6" s="1">
         <v>10046318</v>
@@ -2571,20 +1699,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2811,19 +1939,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D96E9815-3E38-457E-AC60-BC705C73AD1F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3513D4C-5F93-4AB4-B899-280E533C715E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3513D4C-5F93-4AB4-B899-280E533C715E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D96E9815-3E38-457E-AC60-BC705C73AD1F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>